<commit_message>
Maestra oct 2026: Zona Desarrollo (Maryi Castro, 59 clientes) y Meta pasa de Zona Norte a Zona Sur
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Maestra_de_Contactos.xlsx
+++ b/datos/Maestra_de_Contactos.xlsx
@@ -501,7 +501,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -736,12 +736,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G6" t="b">
@@ -769,7 +769,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1981,7 +1981,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2041,7 +2041,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2611,12 +2611,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G38" t="b">
@@ -2644,7 +2644,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -2941,12 +2941,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G44" t="b">
@@ -2974,7 +2974,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -2996,7 +2996,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -3106,12 +3106,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G47" t="b">
@@ -3139,7 +3139,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -3161,12 +3161,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
       <c r="G48" t="b">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
     </row>
@@ -3271,12 +3271,12 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G50" t="b">
@@ -3304,7 +3304,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -3436,7 +3436,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -3546,7 +3546,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -3601,12 +3601,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G56" t="b">
@@ -3634,7 +3634,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -3656,7 +3656,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -3766,12 +3766,12 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G59" t="b">
@@ -3799,7 +3799,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -3986,7 +3986,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -4096,12 +4096,12 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G65" t="b">
@@ -4129,7 +4129,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -4206,12 +4206,12 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G67" t="b">
@@ -4239,7 +4239,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -4261,12 +4261,12 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G68" t="b">
@@ -4294,7 +4294,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -4426,7 +4426,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -4481,12 +4481,12 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G72" t="b">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -4756,7 +4756,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -4811,7 +4811,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -4866,7 +4866,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -4921,7 +4921,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -4976,7 +4976,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -5031,12 +5031,12 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G82" t="b">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -5306,12 +5306,12 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G87" t="b">
@@ -5339,7 +5339,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -5361,7 +5361,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -5416,7 +5416,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -5471,7 +5471,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -5526,12 +5526,12 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G91" t="b">
@@ -5559,7 +5559,7 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -5801,7 +5801,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -5856,7 +5856,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -5911,7 +5911,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -5966,7 +5966,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -6021,7 +6021,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -6076,7 +6076,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -6241,12 +6241,12 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G104" t="b">
@@ -6274,7 +6274,7 @@
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -6351,7 +6351,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -6461,7 +6461,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -6516,7 +6516,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -6571,7 +6571,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -6626,12 +6626,12 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G111" t="b">
@@ -6659,7 +6659,7 @@
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -6736,12 +6736,12 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G113" t="b">
@@ -6769,7 +6769,7 @@
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -6846,7 +6846,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -6901,7 +6901,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -6956,7 +6956,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -7011,7 +7011,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -7121,12 +7121,12 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G120" t="b">
@@ -7154,7 +7154,7 @@
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -7231,7 +7231,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -7341,12 +7341,12 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
       <c r="G124" t="b">
@@ -7374,7 +7374,7 @@
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
     </row>
@@ -7396,7 +7396,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -7506,7 +7506,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -7671,7 +7671,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -7781,12 +7781,12 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G132" t="b">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7946,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -8056,7 +8056,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -8276,12 +8276,12 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G141" t="b">
@@ -8309,7 +8309,7 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -8331,12 +8331,12 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
       <c r="G142" t="b">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="L142" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
     </row>
@@ -8441,7 +8441,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -8496,12 +8496,12 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G145" t="b">
@@ -8529,7 +8529,7 @@
       </c>
       <c r="L145" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -8551,12 +8551,12 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G146" t="b">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="L146" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -8606,12 +8606,12 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
       <c r="G147" t="b">
@@ -8639,7 +8639,7 @@
       </c>
       <c r="L147" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
     </row>
@@ -8936,7 +8936,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -9101,12 +9101,12 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G156" t="b">
@@ -9134,7 +9134,7 @@
       </c>
       <c r="L156" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -9266,12 +9266,12 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G159" t="b">
@@ -9299,7 +9299,7 @@
       </c>
       <c r="L159" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -9926,7 +9926,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
@@ -10036,12 +10036,12 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G173" t="b">
@@ -10069,7 +10069,7 @@
       </c>
       <c r="L173" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -10091,12 +10091,12 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G174" t="b">
@@ -10124,7 +10124,7 @@
       </c>
       <c r="L174" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -10201,7 +10201,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
@@ -10261,7 +10261,7 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
       <c r="G177" t="b">
@@ -10311,12 +10311,12 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G178" t="b">
@@ -10344,7 +10344,7 @@
       </c>
       <c r="L178" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -10421,7 +10421,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
@@ -10476,7 +10476,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -10861,12 +10861,12 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G188" t="b">
@@ -10894,7 +10894,7 @@
       </c>
       <c r="L188" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -10916,12 +10916,12 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G189" t="b">
@@ -10949,7 +10949,7 @@
       </c>
       <c r="L189" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -10971,7 +10971,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
@@ -11026,12 +11026,12 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G191" t="b">
@@ -11059,7 +11059,7 @@
       </c>
       <c r="L191" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -11251,7 +11251,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
@@ -11311,7 +11311,7 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
@@ -11371,7 +11371,7 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
@@ -11431,7 +11431,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
@@ -11551,7 +11551,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
@@ -11666,7 +11666,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
@@ -11901,7 +11901,7 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F206" t="inlineStr">
@@ -12181,12 +12181,12 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G211" t="b">
@@ -12214,7 +12214,7 @@
       </c>
       <c r="L211" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -12291,12 +12291,12 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G213" t="b">
@@ -12324,7 +12324,7 @@
       </c>
       <c r="L213" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -12621,7 +12621,7 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F219" t="inlineStr">
@@ -12676,7 +12676,7 @@
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F220" t="inlineStr">
@@ -12951,7 +12951,7 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
@@ -13061,7 +13061,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
@@ -13396,7 +13396,7 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
@@ -13456,7 +13456,7 @@
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F234" t="inlineStr">
@@ -13516,7 +13516,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
@@ -13576,7 +13576,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
@@ -13696,7 +13696,7 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
@@ -13751,12 +13751,12 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G239" t="b">
@@ -13784,7 +13784,7 @@
       </c>
       <c r="L239" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -13806,12 +13806,12 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G240" t="b">
@@ -13839,7 +13839,7 @@
       </c>
       <c r="L240" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -14161,12 +14161,12 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G246" t="b">
@@ -14194,7 +14194,7 @@
       </c>
       <c r="L246" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -14216,12 +14216,12 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G247" t="b">
@@ -14249,7 +14249,7 @@
       </c>
       <c r="L247" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -14276,7 +14276,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
@@ -14336,7 +14336,7 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
@@ -14516,7 +14516,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
@@ -14631,7 +14631,7 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
@@ -14686,12 +14686,12 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G255" t="b">
@@ -14719,7 +14719,7 @@
       </c>
       <c r="L255" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -14741,7 +14741,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
@@ -14796,7 +14796,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
@@ -15291,7 +15291,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
@@ -15346,12 +15346,12 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
       <c r="G267" t="b">
@@ -15379,7 +15379,7 @@
       </c>
       <c r="L267" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
     </row>
@@ -15401,12 +15401,12 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G268" t="b">
@@ -15434,7 +15434,7 @@
       </c>
       <c r="L268" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -15791,7 +15791,7 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
@@ -15846,12 +15846,12 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
       <c r="G276" t="b">
@@ -15879,7 +15879,7 @@
       </c>
       <c r="L276" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
     </row>
@@ -16441,7 +16441,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
@@ -16666,7 +16666,7 @@
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
@@ -16781,12 +16781,12 @@
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G292" t="b">
@@ -16814,7 +16814,7 @@
       </c>
       <c r="L292" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -16841,7 +16841,7 @@
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
@@ -16961,7 +16961,7 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
@@ -17081,7 +17081,7 @@
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
@@ -17196,12 +17196,12 @@
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G299" t="b">
@@ -17229,7 +17229,7 @@
       </c>
       <c r="L299" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -17366,12 +17366,12 @@
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G302" t="b">
@@ -17399,7 +17399,7 @@
       </c>
       <c r="L302" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -17766,7 +17766,7 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
@@ -17821,7 +17821,7 @@
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
@@ -17876,12 +17876,12 @@
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G311" t="b">
@@ -17909,7 +17909,7 @@
       </c>
       <c r="L311" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -17931,7 +17931,7 @@
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
@@ -18041,7 +18041,7 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
@@ -18096,7 +18096,7 @@
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
@@ -18151,7 +18151,7 @@
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
@@ -18261,7 +18261,7 @@
       </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F318" t="inlineStr">
@@ -18426,12 +18426,12 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G321" t="b">
@@ -18459,7 +18459,7 @@
       </c>
       <c r="L321" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -18481,7 +18481,7 @@
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
@@ -18541,7 +18541,7 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
@@ -18656,7 +18656,7 @@
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
@@ -18716,7 +18716,7 @@
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
@@ -18776,12 +18776,12 @@
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G327" t="b">
@@ -18809,7 +18809,7 @@
       </c>
       <c r="L327" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -18836,7 +18836,7 @@
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
@@ -18896,7 +18896,7 @@
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
@@ -18956,7 +18956,7 @@
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
@@ -19016,7 +19016,7 @@
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
@@ -19371,7 +19371,7 @@
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
@@ -19541,7 +19541,7 @@
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
@@ -19601,7 +19601,7 @@
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F341" t="inlineStr">
@@ -19661,7 +19661,7 @@
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
@@ -19721,7 +19721,7 @@
       </c>
       <c r="E343" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F343" t="inlineStr">
@@ -19781,12 +19781,12 @@
       </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
       <c r="G344" t="b">
@@ -19814,7 +19814,7 @@
       </c>
       <c r="L344" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
     </row>
@@ -19841,7 +19841,7 @@
       </c>
       <c r="E345" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F345" t="inlineStr">
@@ -19901,7 +19901,7 @@
       </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F346" t="inlineStr">
@@ -20251,7 +20251,7 @@
       </c>
       <c r="E352" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F352" t="inlineStr">
@@ -20371,7 +20371,7 @@
       </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F354" t="inlineStr">
@@ -20431,7 +20431,7 @@
       </c>
       <c r="E355" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F355" t="inlineStr">
@@ -20491,7 +20491,7 @@
       </c>
       <c r="E356" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F356" t="inlineStr">
@@ -20611,7 +20611,7 @@
       </c>
       <c r="E358" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F358" t="inlineStr">
@@ -20671,7 +20671,7 @@
       </c>
       <c r="E359" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
@@ -20791,7 +20791,7 @@
       </c>
       <c r="E361" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F361" t="inlineStr">
@@ -20851,7 +20851,7 @@
       </c>
       <c r="E362" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F362" t="inlineStr">
@@ -20971,7 +20971,7 @@
       </c>
       <c r="E364" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F364" t="inlineStr">
@@ -21031,7 +21031,7 @@
       </c>
       <c r="E365" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F365" t="inlineStr">
@@ -21211,7 +21211,7 @@
       </c>
       <c r="E368" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F368" t="inlineStr">
@@ -21271,7 +21271,7 @@
       </c>
       <c r="E369" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F369" t="inlineStr">
@@ -21331,7 +21331,7 @@
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F370" t="inlineStr">
@@ -21391,7 +21391,7 @@
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F371" t="inlineStr">
@@ -21451,7 +21451,7 @@
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F372" t="inlineStr">
@@ -21571,7 +21571,7 @@
       </c>
       <c r="E374" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F374" t="inlineStr">
@@ -21751,7 +21751,7 @@
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F377" t="inlineStr">
@@ -22051,7 +22051,7 @@
       </c>
       <c r="E382" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F382" t="inlineStr">
@@ -22406,7 +22406,7 @@
       </c>
       <c r="E388" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F388" t="inlineStr">
@@ -22571,7 +22571,7 @@
       </c>
       <c r="E391" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F391" t="inlineStr">
@@ -22626,12 +22626,12 @@
       </c>
       <c r="E392" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G392" t="b">
@@ -22659,7 +22659,7 @@
       </c>
       <c r="L392" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -22681,7 +22681,7 @@
       </c>
       <c r="E393" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F393" t="inlineStr">
@@ -22736,7 +22736,7 @@
       </c>
       <c r="E394" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F394" t="inlineStr">
@@ -22791,7 +22791,7 @@
       </c>
       <c r="E395" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F395" t="inlineStr">
@@ -22901,7 +22901,7 @@
       </c>
       <c r="E397" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F397" t="inlineStr">
@@ -22956,7 +22956,7 @@
       </c>
       <c r="E398" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F398" t="inlineStr">
@@ -23011,7 +23011,7 @@
       </c>
       <c r="E399" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F399" t="inlineStr">
@@ -23066,12 +23066,12 @@
       </c>
       <c r="E400" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F400" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G400" t="b">
@@ -23099,7 +23099,7 @@
       </c>
       <c r="L400" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -23121,7 +23121,7 @@
       </c>
       <c r="E401" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F401" t="inlineStr">
@@ -23176,7 +23176,7 @@
       </c>
       <c r="E402" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F402" t="inlineStr">
@@ -23231,7 +23231,7 @@
       </c>
       <c r="E403" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F403" t="inlineStr">
@@ -23286,7 +23286,7 @@
       </c>
       <c r="E404" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F404" t="inlineStr">
@@ -23341,7 +23341,7 @@
       </c>
       <c r="E405" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F405" t="inlineStr">
@@ -23396,7 +23396,7 @@
       </c>
       <c r="E406" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F406" t="inlineStr">
@@ -23451,7 +23451,7 @@
       </c>
       <c r="E407" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F407" t="inlineStr">
@@ -23506,7 +23506,7 @@
       </c>
       <c r="E408" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F408" t="inlineStr">
@@ -23561,7 +23561,7 @@
       </c>
       <c r="E409" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F409" t="inlineStr">
@@ -23616,7 +23616,7 @@
       </c>
       <c r="E410" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F410" t="inlineStr">
@@ -23671,7 +23671,7 @@
       </c>
       <c r="E411" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F411" t="inlineStr">
@@ -23726,7 +23726,7 @@
       </c>
       <c r="E412" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F412" t="inlineStr">
@@ -23781,7 +23781,7 @@
       </c>
       <c r="E413" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F413" t="inlineStr">
@@ -23836,7 +23836,7 @@
       </c>
       <c r="E414" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F414" t="inlineStr">
@@ -23896,7 +23896,7 @@
       </c>
       <c r="E415" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F415" t="inlineStr">
@@ -24016,7 +24016,7 @@
       </c>
       <c r="E417" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F417" t="inlineStr">
@@ -24136,7 +24136,7 @@
       </c>
       <c r="E419" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F419" t="inlineStr">
@@ -24316,7 +24316,7 @@
       </c>
       <c r="E422" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F422" t="inlineStr">
@@ -24436,7 +24436,7 @@
       </c>
       <c r="E424" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F424" t="inlineStr">
@@ -24616,7 +24616,7 @@
       </c>
       <c r="E427" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F427" t="inlineStr">
@@ -25096,7 +25096,7 @@
       </c>
       <c r="E435" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F435" t="inlineStr">
@@ -25151,12 +25151,12 @@
       </c>
       <c r="E436" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F436" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G436" t="b">
@@ -25184,7 +25184,7 @@
       </c>
       <c r="L436" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -25266,12 +25266,12 @@
       </c>
       <c r="E438" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F438" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G438" t="b">
@@ -25299,7 +25299,7 @@
       </c>
       <c r="L438" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -25496,12 +25496,12 @@
       </c>
       <c r="E442" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F442" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G442" t="b">
@@ -25529,7 +25529,7 @@
       </c>
       <c r="L442" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -25551,12 +25551,12 @@
       </c>
       <c r="E443" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F443" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G443" t="b">
@@ -25584,7 +25584,7 @@
       </c>
       <c r="L443" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -25671,7 +25671,7 @@
       </c>
       <c r="E445" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F445" t="inlineStr">
@@ -25911,7 +25911,7 @@
       </c>
       <c r="E449" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F449" t="inlineStr">
@@ -26031,7 +26031,7 @@
       </c>
       <c r="E451" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F451" t="inlineStr">
@@ -26091,7 +26091,7 @@
       </c>
       <c r="E452" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F452" t="inlineStr">
@@ -26151,7 +26151,7 @@
       </c>
       <c r="E453" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F453" t="inlineStr">
@@ -26266,7 +26266,7 @@
       </c>
       <c r="E455" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F455" t="inlineStr">
@@ -26386,7 +26386,7 @@
       </c>
       <c r="E457" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F457" t="inlineStr">
@@ -26506,7 +26506,7 @@
       </c>
       <c r="E459" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F459" t="inlineStr">
@@ -26746,7 +26746,7 @@
       </c>
       <c r="E463" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F463" t="inlineStr">
@@ -26866,7 +26866,7 @@
       </c>
       <c r="E465" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F465" t="inlineStr">
@@ -26986,7 +26986,7 @@
       </c>
       <c r="E467" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F467" t="inlineStr">
@@ -27226,7 +27226,7 @@
       </c>
       <c r="E471" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F471" t="inlineStr">
@@ -27286,7 +27286,7 @@
       </c>
       <c r="E472" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F472" t="inlineStr">
@@ -27346,7 +27346,7 @@
       </c>
       <c r="E473" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F473" t="inlineStr">
@@ -27581,12 +27581,12 @@
       </c>
       <c r="E477" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F477" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
       <c r="G477" t="b">
@@ -27614,7 +27614,7 @@
       </c>
       <c r="L477" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
     </row>
@@ -27641,7 +27641,7 @@
       </c>
       <c r="E478" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F478" t="inlineStr">
@@ -27701,7 +27701,7 @@
       </c>
       <c r="E479" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F479" t="inlineStr">
@@ -27761,7 +27761,7 @@
       </c>
       <c r="E480" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F480" t="inlineStr">
@@ -27821,7 +27821,7 @@
       </c>
       <c r="E481" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F481" t="inlineStr">
@@ -27996,12 +27996,12 @@
       </c>
       <c r="E484" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F484" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G484" t="b">
@@ -28029,7 +28029,7 @@
       </c>
       <c r="L484" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -28056,7 +28056,7 @@
       </c>
       <c r="E485" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F485" t="inlineStr">
@@ -28176,7 +28176,7 @@
       </c>
       <c r="E487" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F487" t="inlineStr">
@@ -28291,12 +28291,12 @@
       </c>
       <c r="E489" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F489" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G489" t="b">
@@ -28324,7 +28324,7 @@
       </c>
       <c r="L489" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -28591,7 +28591,7 @@
       </c>
       <c r="E494" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F494" t="inlineStr">
@@ -28651,7 +28651,7 @@
       </c>
       <c r="E495" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F495" t="inlineStr">
@@ -28711,7 +28711,7 @@
       </c>
       <c r="E496" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F496" t="inlineStr">
@@ -28771,7 +28771,7 @@
       </c>
       <c r="E497" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F497" t="inlineStr">
@@ -28831,7 +28831,7 @@
       </c>
       <c r="E498" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F498" t="inlineStr">
@@ -29061,12 +29061,12 @@
       </c>
       <c r="E502" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F502" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G502" t="b">
@@ -29094,7 +29094,7 @@
       </c>
       <c r="L502" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -29121,7 +29121,7 @@
       </c>
       <c r="E503" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F503" t="inlineStr">
@@ -29241,7 +29241,7 @@
       </c>
       <c r="E505" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F505" t="inlineStr">
@@ -29421,7 +29421,7 @@
       </c>
       <c r="E508" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F508" t="inlineStr">
@@ -29536,7 +29536,7 @@
       </c>
       <c r="E510" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F510" t="inlineStr">
@@ -29596,7 +29596,7 @@
       </c>
       <c r="E511" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F511" t="inlineStr">
@@ -29831,7 +29831,7 @@
       </c>
       <c r="E515" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F515" t="inlineStr">
@@ -29891,7 +29891,7 @@
       </c>
       <c r="E516" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F516" t="inlineStr">
@@ -29951,7 +29951,7 @@
       </c>
       <c r="E517" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F517" t="inlineStr">
@@ -30011,7 +30011,7 @@
       </c>
       <c r="E518" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F518" t="inlineStr">
@@ -30071,7 +30071,7 @@
       </c>
       <c r="E519" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F519" t="inlineStr">
@@ -30131,7 +30131,7 @@
       </c>
       <c r="E520" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F520" t="inlineStr">
@@ -30191,7 +30191,7 @@
       </c>
       <c r="E521" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F521" t="inlineStr">
@@ -30251,12 +30251,12 @@
       </c>
       <c r="E522" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F522" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
       <c r="G522" t="b">
@@ -30284,7 +30284,7 @@
       </c>
       <c r="L522" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
     </row>
@@ -30426,12 +30426,12 @@
       </c>
       <c r="E525" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F525" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
       <c r="G525" t="b">
@@ -30459,7 +30459,7 @@
       </c>
       <c r="L525" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
     </row>
@@ -30481,12 +30481,12 @@
       </c>
       <c r="E526" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F526" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G526" t="b">
@@ -30514,7 +30514,7 @@
       </c>
       <c r="L526" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -30541,7 +30541,7 @@
       </c>
       <c r="E527" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F527" t="inlineStr">
@@ -30716,12 +30716,12 @@
       </c>
       <c r="E530" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F530" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G530" t="b">
@@ -30749,7 +30749,7 @@
       </c>
       <c r="L530" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -30826,7 +30826,7 @@
       </c>
       <c r="E532" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F532" t="inlineStr">
@@ -30881,7 +30881,7 @@
       </c>
       <c r="E533" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F533" t="inlineStr">
@@ -30936,7 +30936,7 @@
       </c>
       <c r="E534" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F534" t="inlineStr">
@@ -31051,12 +31051,12 @@
       </c>
       <c r="E536" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F536" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
       <c r="G536" t="b">
@@ -31084,7 +31084,7 @@
       </c>
       <c r="L536" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
     </row>
@@ -31171,7 +31171,7 @@
       </c>
       <c r="E538" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F538" t="inlineStr">
@@ -31231,7 +31231,7 @@
       </c>
       <c r="E539" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F539" t="inlineStr">
@@ -31291,7 +31291,7 @@
       </c>
       <c r="E540" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F540" t="inlineStr">
@@ -31526,12 +31526,12 @@
       </c>
       <c r="E544" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F544" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
       <c r="G544" t="b">
@@ -31559,7 +31559,7 @@
       </c>
       <c r="L544" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
     </row>
@@ -31586,7 +31586,7 @@
       </c>
       <c r="E545" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F545" t="inlineStr">
@@ -31646,12 +31646,12 @@
       </c>
       <c r="E546" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F546" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G546" t="b">
@@ -31679,7 +31679,7 @@
       </c>
       <c r="L546" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -31821,12 +31821,12 @@
       </c>
       <c r="E549" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F549" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G549" t="b">
@@ -31854,7 +31854,7 @@
       </c>
       <c r="L549" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -31876,12 +31876,12 @@
       </c>
       <c r="E550" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F550" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G550" t="b">
@@ -31909,7 +31909,7 @@
       </c>
       <c r="L550" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -31931,7 +31931,7 @@
       </c>
       <c r="E551" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F551" t="inlineStr">
@@ -32111,12 +32111,12 @@
       </c>
       <c r="E554" t="inlineStr">
         <is>
-          <t>Lizeth Geraldine Ramos Guerrero</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F554" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
       <c r="G554" t="b">
@@ -32144,7 +32144,7 @@
       </c>
       <c r="L554" t="inlineStr">
         <is>
-          <t>Zona Norte</t>
+          <t>Zona Sur</t>
         </is>
       </c>
     </row>
@@ -32346,7 +32346,7 @@
       </c>
       <c r="E558" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F558" t="inlineStr">
@@ -32401,7 +32401,7 @@
       </c>
       <c r="E559" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F559" t="inlineStr">
@@ -32461,7 +32461,7 @@
       </c>
       <c r="E560" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F560" t="inlineStr">
@@ -32521,7 +32521,7 @@
       </c>
       <c r="E561" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F561" t="inlineStr">
@@ -32701,7 +32701,7 @@
       </c>
       <c r="E564" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F564" t="inlineStr">
@@ -32761,7 +32761,7 @@
       </c>
       <c r="E565" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F565" t="inlineStr">
@@ -32871,7 +32871,7 @@
       </c>
       <c r="E567" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F567" t="inlineStr">
@@ -32931,7 +32931,7 @@
       </c>
       <c r="E568" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F568" t="inlineStr">
@@ -33051,7 +33051,7 @@
       </c>
       <c r="E570" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F570" t="inlineStr">
@@ -33171,7 +33171,7 @@
       </c>
       <c r="E572" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F572" t="inlineStr">
@@ -33231,12 +33231,12 @@
       </c>
       <c r="E573" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Maryi Tatiana Castro Castañeda</t>
         </is>
       </c>
       <c r="F573" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
       <c r="G573" t="b">
@@ -33264,7 +33264,7 @@
       </c>
       <c r="L573" t="inlineStr">
         <is>
-          <t>Zona Sur</t>
+          <t>Zona Desarrollo</t>
         </is>
       </c>
     </row>
@@ -33411,7 +33411,7 @@
       </c>
       <c r="E576" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F576" t="inlineStr">
@@ -33471,7 +33471,7 @@
       </c>
       <c r="E577" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F577" t="inlineStr">
@@ -33591,7 +33591,7 @@
       </c>
       <c r="E579" t="inlineStr">
         <is>
-          <t>Vacante Epithelium</t>
+          <t>Yunelis Esther Caballero Anillo</t>
         </is>
       </c>
       <c r="F579" t="inlineStr">

</xml_diff>